<commit_message>
Timesheet AdTech Oct 2026: revise second tasks for 5 single-task roles
No CAPEX borrowed from other catalog roles (September had none). Director ->
250 business customers, Gryada -> 226 data migration, Klimenko -> OPEX 221
production support of ad serving instead of a product manager's CAPEX task.
Check script now fails on cross-role CAPEX.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WUQDQoJZYHaVzbkcZbnkgZ
</commit_message>
<xml_diff>
--- a/out/Таймшит_AdTech_октябрь_2026_заполнен.xlsx
+++ b/out/Таймшит_AdTech_октябрь_2026_заполнен.xlsx
@@ -14476,29 +14476,29 @@
       </c>
       <c r="R139" s="8" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="S139" s="8" t="inlineStr">
         <is>
-          <t>Интеграция ПО</t>
+          <t>Разработка (кодирование) ПО</t>
         </is>
       </c>
       <c r="T139" s="8" t="inlineStr">
         <is>
-          <t>Дедупликация событий показов и кликов: приемка функциональности и подготовка к запуску</t>
+          <t>Сопровождение промышленной эксплуатации показа рекламы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="U139" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-202</t>
+          <t>ADTHPL-221</t>
         </is>
       </c>
       <c r="V139" s="25" t="n">
         <v>46296</v>
       </c>
       <c r="W139" s="25" t="n">
-        <v>46311</v>
+        <v>46318</v>
       </c>
       <c r="X139" s="8" t="n"/>
     </row>
@@ -21714,12 +21714,12 @@
       </c>
       <c r="T211" s="8" t="inlineStr">
         <is>
-          <t>Исправление дефектов промышленной эксплуатации показа рекламы (4 кв. 2026)</t>
+          <t>Миграция и перенос данных между хранилищами (4 кв. 2026)</t>
         </is>
       </c>
       <c r="U211" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-222</t>
+          <t>ADTHPL-226</t>
         </is>
       </c>
       <c r="V211" s="25" t="n">
@@ -22110,12 +22110,12 @@
       </c>
       <c r="T215" s="8" t="inlineStr">
         <is>
-          <t>Управление портфелем разработки и бюджетом управления (4 кв. 2026)</t>
+          <t>Взаимодействие с бизнес-заказчиками и приоритизация бэклога (4 кв. 2026)</t>
         </is>
       </c>
       <c r="U215" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-249</t>
+          <t>ADTHPL-250</t>
         </is>
       </c>
       <c r="V215" s="25" t="n">
@@ -25311,7 +25311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I243"/>
+  <dimension ref="A1:I240"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -27575,13 +27575,13 @@
         <v>136</v>
       </c>
       <c r="E69" t="n">
-        <v>136</v>
+        <v>96</v>
       </c>
       <c r="F69" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="G69" t="n">
-        <v>1</v>
+        <v>0.706</v>
       </c>
       <c r="H69" t="n">
         <v>2</v>
@@ -30441,12 +30441,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ADTHPL-202</t>
+          <t>ADTHPL-203</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Дедупликация событий показов и кликов: приемка функциональности и подготовка к запуску</t>
+          <t>Управление согласиями пользователей на обработку данных: анализ данных и проектирование метрик</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -30456,28 +30456,28 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Менеджер продукта</t>
+          <t>Аналитик данных</t>
         </is>
       </c>
       <c r="E161" t="n">
-        <v>40</v>
+        <v>96</v>
       </c>
       <c r="F161" t="n">
         <v>1</v>
       </c>
       <c r="G161" t="n">
-        <v>310</v>
+        <v>254</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ADTHPL-203</t>
+          <t>ADTHPL-204</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: анализ данных и проектирование метрик</t>
+          <t>Управление согласиями пользователей на обработку данных: спецификация форматов обмена данными</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -30491,24 +30491,24 @@
         </is>
       </c>
       <c r="E162" t="n">
-        <v>96</v>
+        <v>280</v>
       </c>
       <c r="F162" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G162" t="n">
-        <v>254</v>
+        <v>70</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>ADTHPL-204</t>
+          <t>ADTHPL-205</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: спецификация форматов обмена данными</t>
+          <t>Управление согласиями пользователей на обработку данных: проектирование модели данных</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -30518,28 +30518,28 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Аналитик данных</t>
+          <t>Ведущий аналитик данных</t>
         </is>
       </c>
       <c r="E163" t="n">
-        <v>280</v>
+        <v>120</v>
       </c>
       <c r="F163" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G163" t="n">
-        <v>70</v>
+        <v>230</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ADTHPL-205</t>
+          <t>ADTHPL-206</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: проектирование модели данных</t>
+          <t>Управление согласиями пользователей на обработку данных: разработка требований и спецификации интеграций</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -30549,28 +30549,28 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Ведущий аналитик данных</t>
+          <t>Системный аналитик</t>
         </is>
       </c>
       <c r="E164" t="n">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="F164" t="n">
         <v>1</v>
       </c>
       <c r="G164" t="n">
-        <v>230</v>
+        <v>262</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ADTHPL-206</t>
+          <t>ADTHPL-207</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: разработка требований и спецификации интеграций</t>
+          <t>Управление согласиями пользователей на обработку данных: проектирование архитектуры решения</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -30596,12 +30596,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ADTHPL-207</t>
+          <t>ADTHPL-208</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: проектирование архитектуры решения</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование интерфейса и прототипирование</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -30611,28 +30611,28 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Системный аналитик</t>
+          <t>Дизайнер продукта</t>
         </is>
       </c>
       <c r="E166" t="n">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="F166" t="n">
         <v>1</v>
       </c>
       <c r="G166" t="n">
-        <v>262</v>
+        <v>302</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ADTHPL-208</t>
+          <t>ADTHPL-209</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование интерфейса и прототипирование</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: макеты экранов и дизайн-система</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -30646,24 +30646,24 @@
         </is>
       </c>
       <c r="E167" t="n">
-        <v>48</v>
+        <v>128</v>
       </c>
       <c r="F167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G167" t="n">
-        <v>302</v>
+        <v>222</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ADTHPL-209</t>
+          <t>ADTHPL-210</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: макеты экранов и дизайн-система</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование пользовательских сценариев</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -30677,24 +30677,24 @@
         </is>
       </c>
       <c r="E168" t="n">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="F168" t="n">
         <v>2</v>
       </c>
       <c r="G168" t="n">
-        <v>222</v>
+        <v>238</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ADTHPL-210</t>
+          <t>ADTHPL-211</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование пользовательских сценариев</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: адаптивные макеты для мобильных устройств</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -30720,12 +30720,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ADTHPL-211</t>
+          <t>ADTHPL-212</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: адаптивные макеты для мобильных устройств</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование пользовательских сценариев, итерация 2</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -30739,24 +30739,24 @@
         </is>
       </c>
       <c r="E170" t="n">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="F170" t="n">
         <v>2</v>
       </c>
       <c r="G170" t="n">
-        <v>238</v>
+        <v>222</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ADTHPL-212</t>
+          <t>ADTHPL-213</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование пользовательских сценариев, итерация 2</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: юзабилити-тестирование интерфейса</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -30766,28 +30766,28 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Дизайнер продукта</t>
+          <t>Исследователь пользовательского опыта</t>
         </is>
       </c>
       <c r="E171" t="n">
-        <v>128</v>
+        <v>80</v>
       </c>
       <c r="F171" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G171" t="n">
-        <v>222</v>
+        <v>270</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>ADTHPL-213</t>
+          <t>ADTHPL-214</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: юзабилити-тестирование интерфейса</t>
+          <t>Отчет sales lift по рекламной кампании: анализ данных и проектирование метрик</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -30797,28 +30797,28 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Исследователь пользовательского опыта</t>
+          <t>Аналитик данных</t>
         </is>
       </c>
       <c r="E172" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="F172" t="n">
         <v>1</v>
       </c>
       <c r="G172" t="n">
-        <v>270</v>
+        <v>230</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ADTHPL-214</t>
+          <t>ADTHPL-215</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Отчет sales lift по рекламной кампании: анализ данных и проектирование метрик</t>
+          <t>Отчет sales lift по рекламной кампании: анализ источников и качества данных</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -30844,12 +30844,12 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ADTHPL-215</t>
+          <t>ADTHPL-216</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Отчет sales lift по рекламной кампании: анализ источников и качества данных</t>
+          <t>Отчет sales lift по рекламной кампании: спецификация форматов обмена данными</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -30859,7 +30859,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Аналитик данных</t>
+          <t>Ведущий аналитик данных</t>
         </is>
       </c>
       <c r="E174" t="n">
@@ -30875,12 +30875,12 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ADTHPL-216</t>
+          <t>ADTHPL-217</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Отчет sales lift по рекламной кампании: спецификация форматов обмена данными</t>
+          <t>Кабинет партнера: ссылки, промокоды, статистика: функциональное и интеграционное тестирование</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -30890,28 +30890,28 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Ведущий аналитик данных</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E175" t="n">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="F175" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G175" t="n">
-        <v>230</v>
+        <v>190</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ADTHPL-217</t>
+          <t>ADTHPL-218</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Кабинет партнера: ссылки, промокоды, статистика: функциональное и интеграционное тестирование</t>
+          <t>Кабинет партнера: ссылки, промокоды, статистика: нагрузочное тестирование</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -30925,24 +30925,24 @@
         </is>
       </c>
       <c r="E176" t="n">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="F176" t="n">
         <v>2</v>
       </c>
       <c r="G176" t="n">
-        <v>190</v>
+        <v>198</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ADTHPL-218</t>
+          <t>ADTHPL-219</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Кабинет партнера: ссылки, промокоды, статистика: нагрузочное тестирование</t>
+          <t>Кабинет партнера: ссылки, промокоды, статистика: автоматизация регрессионных тестов</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -30956,24 +30956,24 @@
         </is>
       </c>
       <c r="E177" t="n">
-        <v>152</v>
+        <v>192</v>
       </c>
       <c r="F177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G177" t="n">
-        <v>198</v>
+        <v>158</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ADTHPL-219</t>
+          <t>ADTHPL-220</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Кабинет партнера: ссылки, промокоды, статистика: автоматизация регрессионных тестов</t>
+          <t>Кабинет партнера: ссылки, промокоды, статистика: тестирование отказоустойчивости</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -30987,55 +30987,55 @@
         </is>
       </c>
       <c r="E178" t="n">
-        <v>192</v>
+        <v>112</v>
       </c>
       <c r="F178" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G178" t="n">
-        <v>158</v>
+        <v>238</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ADTHPL-220</t>
+          <t>ADTHPL-221</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Кабинет партнера: ссылки, промокоды, статистика: тестирование отказоустойчивости</t>
+          <t>Сопровождение промышленной эксплуатации показа рекламы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Ведущий инженер сопровождения</t>
         </is>
       </c>
       <c r="E179" t="n">
-        <v>112</v>
+        <v>342</v>
       </c>
       <c r="F179" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G179" t="n">
-        <v>238</v>
+        <v>8</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ADTHPL-221</t>
+          <t>ADTHPL-224</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации показа рекламы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Административное управление командой показа рекламы: планирование, найм, оценка (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -31045,28 +31045,28 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Ведущий инженер сопровождения</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E180" t="n">
-        <v>302</v>
+        <v>350</v>
       </c>
       <c r="F180" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G180" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ADTHPL-222</t>
+          <t>ADTHPL-225</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Исправление дефектов промышленной эксплуатации показа рекламы (4 кв. 2026)</t>
+          <t>Сопровождение промышленной эксплуатации сбора событий: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -31076,28 +31076,28 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Ведущий инженер сопровождения</t>
         </is>
       </c>
       <c r="E181" t="n">
-        <v>56</v>
+        <v>146</v>
       </c>
       <c r="F181" t="n">
         <v>1</v>
       </c>
       <c r="G181" t="n">
-        <v>294</v>
+        <v>204</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ADTHPL-224</t>
+          <t>ADTHPL-226</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Административное управление командой показа рекламы: планирование, найм, оценка (4 кв. 2026)</t>
+          <t>Миграция и перенос данных между хранилищами (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -31107,28 +31107,28 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E182" t="n">
-        <v>350</v>
+        <v>56</v>
       </c>
       <c r="F182" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G182" t="n">
-        <v>0</v>
+        <v>294</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ADTHPL-225</t>
+          <t>ADTHPL-227</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации сбора событий: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Административное управление командой сбора событий: планирование, найм, оценка (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -31138,28 +31138,28 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Ведущий инженер сопровождения</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E183" t="n">
-        <v>146</v>
+        <v>246</v>
       </c>
       <c r="F183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G183" t="n">
-        <v>204</v>
+        <v>104</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>ADTHPL-226</t>
+          <t>ADTHPL-228</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Миграция и перенос данных между хранилищами (4 кв. 2026)</t>
+          <t>Сопровождение промышленной эксплуатации рекламного кабинета: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -31169,28 +31169,28 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Ведущий инженер сопровождения</t>
         </is>
       </c>
       <c r="E184" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F184" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G184" t="n">
-        <v>350</v>
+        <v>286</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ADTHPL-227</t>
+          <t>ADTHPL-230</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Административное управление командой сбора событий: планирование, найм, оценка (4 кв. 2026)</t>
+          <t>Административное управление командой рекламного кабинета: планирование, найм, оценка (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -31204,24 +31204,24 @@
         </is>
       </c>
       <c r="E185" t="n">
-        <v>246</v>
+        <v>218</v>
       </c>
       <c r="F185" t="n">
         <v>2</v>
       </c>
       <c r="G185" t="n">
-        <v>104</v>
+        <v>132</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ADTHPL-228</t>
+          <t>ADTHPL-233</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации рекламного кабинета: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Сопровождение промышленной эксплуатации аналитики: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -31235,24 +31235,24 @@
         </is>
       </c>
       <c r="E186" t="n">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="F186" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G186" t="n">
-        <v>286</v>
+        <v>254</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ADTHPL-229</t>
+          <t>ADTHPL-234</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Снижение технического долга и обновление зависимостей (4 кв. 2026)</t>
+          <t>Административное управление командой аналитики: планирование, найм, оценка (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -31262,28 +31262,28 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Главный разработчик</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E187" t="n">
-        <v>0</v>
+        <v>218</v>
       </c>
       <c r="F187" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G187" t="n">
-        <v>350</v>
+        <v>132</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ADTHPL-230</t>
+          <t>ADTHPL-235</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Административное управление командой рекламного кабинета: планирование, найм, оценка (4 кв. 2026)</t>
+          <t>Сопровождение промышленной эксплуатации партнерской платформы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -31293,28 +31293,28 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Инженер сопровождения</t>
         </is>
       </c>
       <c r="E188" t="n">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="F188" t="n">
         <v>2</v>
       </c>
       <c r="G188" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ADTHPL-233</t>
+          <t>ADTHPL-236</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации аналитики: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Административное управление командой партнерской платформы: планирование, найм, оценка (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -31324,28 +31324,28 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Ведущий инженер сопровождения</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E189" t="n">
-        <v>96</v>
+        <v>210</v>
       </c>
       <c r="F189" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G189" t="n">
-        <v>254</v>
+        <v>140</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ADTHPL-234</t>
+          <t>ADTHPL-237</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Административное управление командой аналитики: планирование, найм, оценка (4 кв. 2026)</t>
+          <t>Сопровождение промышленной эксплуатации интеграции с ОРД: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -31355,28 +31355,28 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Инженер сопровождения</t>
         </is>
       </c>
       <c r="E190" t="n">
-        <v>218</v>
+        <v>96</v>
       </c>
       <c r="F190" t="n">
         <v>2</v>
       </c>
       <c r="G190" t="n">
-        <v>132</v>
+        <v>254</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ADTHPL-235</t>
+          <t>ADTHPL-238</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации партнерской платформы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Административное управление командой интеграции с ОРД: планирование, найм, оценка (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -31386,28 +31386,28 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Инженер сопровождения</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E191" t="n">
-        <v>216</v>
+        <v>123</v>
       </c>
       <c r="F191" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G191" t="n">
-        <v>134</v>
+        <v>227</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ADTHPL-236</t>
+          <t>ADTHPL-239</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Административное управление командой партнерской платформы: планирование, найм, оценка (4 кв. 2026)</t>
+          <t>Сопровождение регулярной отчетности Эдтех: доработки и разбор обращений (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -31417,28 +31417,28 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Ведущий разработчик проекта Эдтех</t>
         </is>
       </c>
       <c r="E192" t="n">
-        <v>210</v>
+        <v>120</v>
       </c>
       <c r="F192" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G192" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>ADTHPL-237</t>
+          <t>ADTHPL-242</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации интеграции с ОРД: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Стратегическое управление департаментом и бюджетирование (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -31448,28 +31448,28 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Инженер сопровождения</t>
+          <t>Директор департамента</t>
         </is>
       </c>
       <c r="E193" t="n">
-        <v>96</v>
+        <v>120</v>
       </c>
       <c r="F193" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G193" t="n">
-        <v>254</v>
+        <v>230</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ADTHPL-238</t>
+          <t>ADTHPL-243</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Административное управление командой интеграции с ОРД: планирование, найм, оценка (4 кв. 2026)</t>
+          <t>Исследование рынка и конкурентных рекламных решений (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -31479,28 +31479,28 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Менеджер продукта</t>
         </is>
       </c>
       <c r="E194" t="n">
-        <v>123</v>
+        <v>210</v>
       </c>
       <c r="F194" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G194" t="n">
-        <v>227</v>
+        <v>140</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ADTHPL-239</t>
+          <t>ADTHPL-244</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Сопровождение регулярной отчетности Эдтех: доработки и разбор обращений (4 кв. 2026)</t>
+          <t>Управление графиком проектов платформы: сроки, риски, статус-отчетность (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -31510,28 +31510,28 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Ведущий разработчик проекта Эдтех</t>
+          <t>Менеджер проектов</t>
         </is>
       </c>
       <c r="E195" t="n">
-        <v>120</v>
+        <v>125.3</v>
       </c>
       <c r="F195" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G195" t="n">
-        <v>230</v>
+        <v>224.7</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ADTHPL-242</t>
+          <t>ADTHPL-245</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Стратегическое управление департаментом и бюджетирование (4 кв. 2026)</t>
+          <t>Участие в найме и онбординге сотрудников платформы (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -31541,28 +31541,28 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Директор департамента</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E196" t="n">
-        <v>120</v>
+        <v>27</v>
       </c>
       <c r="F196" t="n">
         <v>1</v>
       </c>
       <c r="G196" t="n">
-        <v>230</v>
+        <v>323</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>ADTHPL-243</t>
+          <t>ADTHPL-246</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Исследование рынка и конкурентных рекламных решений (4 кв. 2026)</t>
+          <t>Планирование ресурсов и отчетность направления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -31572,28 +31572,28 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Менеджер продукта</t>
+          <t>Руководитель направления</t>
         </is>
       </c>
       <c r="E197" t="n">
-        <v>210</v>
+        <v>176</v>
       </c>
       <c r="F197" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G197" t="n">
-        <v>140</v>
+        <v>174</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ADTHPL-244</t>
+          <t>ADTHPL-247</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Управление графиком проектов платформы: сроки, риски, статус-отчетность (4 кв. 2026)</t>
+          <t>Развитие компетенций и процессов направления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -31603,28 +31603,28 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Менеджер проектов</t>
+          <t>Руководитель направления</t>
         </is>
       </c>
       <c r="E198" t="n">
-        <v>125.3</v>
+        <v>176</v>
       </c>
       <c r="F198" t="n">
         <v>2</v>
       </c>
       <c r="G198" t="n">
-        <v>224.7</v>
+        <v>174</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ADTHPL-245</t>
+          <t>ADTHPL-248</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Участие в найме и онбординге сотрудников платформы (4 кв. 2026)</t>
+          <t>Координация межкомандных проектов и коммуникация с заказчиками (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -31634,28 +31634,28 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Руководитель проектов</t>
         </is>
       </c>
       <c r="E199" t="n">
-        <v>27</v>
+        <v>68.3</v>
       </c>
       <c r="F199" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G199" t="n">
-        <v>323</v>
+        <v>281.7</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ADTHPL-246</t>
+          <t>ADTHPL-249</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Планирование ресурсов и отчетность направления (4 кв. 2026)</t>
+          <t>Управление портфелем разработки и бюджетом управления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -31665,28 +31665,28 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Руководитель направления</t>
+          <t>Руководитель управления</t>
         </is>
       </c>
       <c r="E200" t="n">
-        <v>176</v>
+        <v>288</v>
       </c>
       <c r="F200" t="n">
         <v>2</v>
       </c>
       <c r="G200" t="n">
-        <v>174</v>
+        <v>62</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ADTHPL-247</t>
+          <t>ADTHPL-250</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Развитие компетенций и процессов направления (4 кв. 2026)</t>
+          <t>Взаимодействие с бизнес-заказчиками и приоритизация бэклога (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -31696,28 +31696,28 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Руководитель направления</t>
+          <t>Руководитель управления</t>
         </is>
       </c>
       <c r="E201" t="n">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="F201" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G201" t="n">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>ADTHPL-248</t>
+          <t>ADTHPL-251</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Координация межкомандных проектов и коммуникация с заказчиками (4 кв. 2026)</t>
+          <t>Планирование численности и развитие команд управления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -31727,121 +31727,121 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>Руководитель проектов</t>
+          <t>Руководитель управления</t>
         </is>
       </c>
       <c r="E202" t="n">
-        <v>68.3</v>
+        <v>112</v>
       </c>
       <c r="F202" t="n">
         <v>2</v>
       </c>
       <c r="G202" t="n">
-        <v>281.7</v>
+        <v>238</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>ADTHPL-249</t>
+          <t>ADTHPL-253</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Управление портфелем разработки и бюджетом управления (4 кв. 2026)</t>
+          <t>Геораспределенная отказоустойчивая инфраструктура выдачи: функциональное и интеграционное тестирование</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Руководитель управления</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E203" t="n">
-        <v>344</v>
+        <v>160</v>
       </c>
       <c r="F203" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G203" t="n">
-        <v>6</v>
+        <v>190</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>ADTHPL-250</t>
+          <t>ADTHPL-254</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Взаимодействие с бизнес-заказчиками и приоритизация бэклога (4 кв. 2026)</t>
+          <t>Бюджет и биллинг рекламодателя в кабинете: функциональное и интеграционное тестирование</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>Руководитель управления</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E204" t="n">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="F204" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G204" t="n">
-        <v>222</v>
+        <v>230</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>ADTHPL-251</t>
+          <t>ADTHPL-255</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Планирование численности и развитие команд управления (4 кв. 2026)</t>
+          <t>Модерация креативов в рекламном кабинете: разработка серверной части и API</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>Руководитель управления</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E205" t="n">
-        <v>112</v>
+        <v>56</v>
       </c>
       <c r="F205" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G205" t="n">
-        <v>238</v>
+        <v>294</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>ADTHPL-253</t>
+          <t>ADTHPL-256</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Геораспределенная отказоустойчивая инфраструктура выдачи: функциональное и интеграционное тестирование</t>
+          <t>Модерация креативов в рекламном кабинете: разработка пользовательского интерфейса</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -31851,90 +31851,90 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Разработчик</t>
         </is>
       </c>
       <c r="E206" t="n">
-        <v>160</v>
+        <v>56</v>
       </c>
       <c r="F206" t="n">
         <v>1</v>
       </c>
       <c r="G206" t="n">
-        <v>190</v>
+        <v>294</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>ADTHPL-254</t>
+          <t>ADTHPL-257</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Бюджет и биллинг рекламодателя в кабинете: функциональное и интеграционное тестирование</t>
+          <t>Аукцион первой цены с корректировкой ставок: исследование и формирование продуктовой гипотезы</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Ведущий менеджер продукта</t>
         </is>
       </c>
       <c r="E207" t="n">
-        <v>120</v>
+        <v>140</v>
       </c>
       <c r="F207" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G207" t="n">
-        <v>230</v>
+        <v>210</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>ADTHPL-255</t>
+          <t>ADTHPL-258</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Модерация креативов в рекламном кабинете: разработка серверной части и API</t>
+          <t>Аукцион первой цены с корректировкой ставок: оценка эффекта и подготовка бизнес-кейса</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Менеджер продукта</t>
         </is>
       </c>
       <c r="E208" t="n">
-        <v>56</v>
+        <v>210</v>
       </c>
       <c r="F208" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G208" t="n">
-        <v>294</v>
+        <v>140</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>ADTHPL-256</t>
+          <t>ADTHPL-259</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Модерация креативов в рекламном кабинете: разработка пользовательского интерфейса</t>
+          <t>Прогноз кликабельности для ранжирования ставок: функциональное и интеграционное тестирование</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -31944,90 +31944,90 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Разработчик</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E209" t="n">
-        <v>56</v>
+        <v>120</v>
       </c>
       <c r="F209" t="n">
         <v>1</v>
       </c>
       <c r="G209" t="n">
-        <v>294</v>
+        <v>230</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>ADTHPL-257</t>
+          <t>ADTHPL-260</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Аукцион первой цены с корректировкой ставок: исследование и формирование продуктовой гипотезы</t>
+          <t>Прогноз кликабельности для ранжирования ставок: нагрузочное тестирование</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Ведущий менеджер продукта</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E210" t="n">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="F210" t="n">
         <v>2</v>
       </c>
       <c r="G210" t="n">
-        <v>210</v>
+        <v>238</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>ADTHPL-258</t>
+          <t>ADTHPL-261</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Аукцион первой цены с корректировкой ставок: оценка эффекта и подготовка бизнес-кейса</t>
+          <t>Прогноз кликабельности для ранжирования ставок: автоматизация регрессионных тестов</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>Менеджер продукта</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E211" t="n">
-        <v>210</v>
+        <v>120</v>
       </c>
       <c r="F211" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G211" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>ADTHPL-259</t>
+          <t>ADTHPL-262</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Прогноз кликабельности для ранжирования ставок: функциональное и интеграционное тестирование</t>
+          <t>Прогноз кликабельности для ранжирования ставок: тестирование отказоустойчивости</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -32037,7 +32037,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Главный специалист по тестированию</t>
         </is>
       </c>
       <c r="E212" t="n">
@@ -32053,12 +32053,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>ADTHPL-260</t>
+          <t>ADTHPL-263</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Прогноз кликабельности для ранжирования ставок: нагрузочное тестирование</t>
+          <t>Прогноз кликабельности для ранжирования ставок: тестирование безопасности</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -32068,28 +32068,28 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Главный специалист по тестированию</t>
         </is>
       </c>
       <c r="E213" t="n">
-        <v>112</v>
+        <v>176</v>
       </c>
       <c r="F213" t="n">
         <v>2</v>
       </c>
       <c r="G213" t="n">
-        <v>238</v>
+        <v>174</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>ADTHPL-261</t>
+          <t>ADTHPL-264</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Прогноз кликабельности для ранжирования ставок: автоматизация регрессионных тестов</t>
+          <t>Таргетинг по сегментам аудиторий в реальном времени: проектирование архитектуры и разработка ядра</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -32099,28 +32099,28 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Главный разработчик</t>
         </is>
       </c>
       <c r="E214" t="n">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="F214" t="n">
         <v>1</v>
       </c>
       <c r="G214" t="n">
-        <v>230</v>
+        <v>270</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>ADTHPL-262</t>
+          <t>ADTHPL-265</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Прогноз кликабельности для ранжирования ставок: тестирование отказоустойчивости</t>
+          <t>Мастер создания кампании в рекламном кабинете: функциональное и интеграционное тестирование</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -32130,28 +32130,28 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>Главный специалист по тестированию</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E215" t="n">
-        <v>120</v>
+        <v>152</v>
       </c>
       <c r="F215" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G215" t="n">
-        <v>230</v>
+        <v>198</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>ADTHPL-263</t>
+          <t>ADTHPL-266</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Прогноз кликабельности для ранжирования ставок: тестирование безопасности</t>
+          <t>Мастер создания кампании в рекламном кабинете: тестирование отказоустойчивости</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -32161,28 +32161,28 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>Главный специалист по тестированию</t>
+          <t>Ведущий специалист по тестированию</t>
         </is>
       </c>
       <c r="E216" t="n">
-        <v>176</v>
+        <v>88</v>
       </c>
       <c r="F216" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G216" t="n">
-        <v>174</v>
+        <v>262</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>ADTHPL-264</t>
+          <t>ADTHPL-267</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Таргетинг по сегментам аудиторий в реальном времени: проектирование архитектуры и разработка ядра</t>
+          <t>Мастер создания кампании в рекламном кабинете: нагрузочное тестирование</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -32192,28 +32192,28 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>Главный разработчик</t>
+          <t>Главный специалист по тестированию</t>
         </is>
       </c>
       <c r="E217" t="n">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="F217" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G217" t="n">
-        <v>270</v>
+        <v>150</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>ADTHPL-265</t>
+          <t>ADTHPL-268</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Мастер создания кампании в рекламном кабинете: функциональное и интеграционное тестирование</t>
+          <t>Мастер создания кампании в рекламном кабинете: тестирование безопасности</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -32223,7 +32223,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Главный специалист по тестированию</t>
         </is>
       </c>
       <c r="E218" t="n">
@@ -32239,12 +32239,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>ADTHPL-266</t>
+          <t>ADTHPL-269</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Мастер создания кампании в рекламном кабинете: тестирование отказоустойчивости</t>
+          <t>Мастер создания кампании в рекламном кабинете: автоматизация регрессионных тестов</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -32254,28 +32254,28 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>Ведущий специалист по тестированию</t>
+          <t>Специалист по тестированию</t>
         </is>
       </c>
       <c r="E219" t="n">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="F219" t="n">
         <v>1</v>
       </c>
       <c r="G219" t="n">
-        <v>262</v>
+        <v>230</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ADTHPL-267</t>
+          <t>ADTHPL-270</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Мастер создания кампании в рекламном кабинете: нагрузочное тестирование</t>
+          <t>Мастер создания кампании в рекламном кабинете: приемочное тестирование с бизнесом</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -32285,28 +32285,28 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>Главный специалист по тестированию</t>
+          <t>Специалист по тестированию</t>
         </is>
       </c>
       <c r="E220" t="n">
-        <v>200</v>
+        <v>56</v>
       </c>
       <c r="F220" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G220" t="n">
-        <v>150</v>
+        <v>294</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ADTHPL-268</t>
+          <t>ADTHPL-271</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Мастер создания кампании в рекламном кабинете: тестирование безопасности</t>
+          <t>Автоматическая передача в ОРД данных о показах и актах: разработка серверной части и API</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -32316,28 +32316,28 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>Главный специалист по тестированию</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E221" t="n">
-        <v>152</v>
+        <v>0</v>
       </c>
       <c r="F221" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G221" t="n">
-        <v>198</v>
+        <v>350</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>ADTHPL-269</t>
+          <t>ADTHPL-272</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Мастер создания кампании в рекламном кабинете: автоматизация регрессионных тестов</t>
+          <t>Автоматическая передача в ОРД данных о показах и актах: мониторинг и логирование новой функциональности</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -32347,28 +32347,28 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>Специалист по тестированию</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E222" t="n">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F222" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G222" t="n">
-        <v>230</v>
+        <v>350</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>ADTHPL-270</t>
+          <t>ADTHPL-273</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Мастер создания кампании в рекламном кабинете: приемочное тестирование с бизнесом</t>
+          <t>Интеграция с внешними SSP по OpenRTB 2.6: разработка серверной части и API</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -32378,28 +32378,28 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Специалист по тестированию</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E223" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="F223" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G223" t="n">
-        <v>294</v>
+        <v>350</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>ADTHPL-271</t>
+          <t>ADTHPL-274</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Автоматическая передача в ОРД данных о показах и актах: разработка серверной части и API</t>
+          <t>Интеграция с внешними SSP по OpenRTB 2.6: разработка пользовательского интерфейса</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -32425,12 +32425,12 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>ADTHPL-272</t>
+          <t>ADTHPL-275</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Автоматическая передача в ОРД данных о показах и актах: мониторинг и логирование новой функциональности</t>
+          <t>Интеграция с внешними SSP по OpenRTB 2.6: интеграция со смежными модулями платформы</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -32456,12 +32456,12 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>ADTHPL-273</t>
+          <t>ADTHPL-276</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Интеграция с внешними SSP по OpenRTB 2.6: разработка серверной части и API</t>
+          <t>Интеграция с внешними SSP по OpenRTB 2.6: разработка хранения и обработки данных</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -32487,12 +32487,12 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>ADTHPL-274</t>
+          <t>ADTHPL-277</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Интеграция с внешними SSP по OpenRTB 2.6: разработка пользовательского интерфейса</t>
+          <t>Интеграция с внешними SSP по OpenRTB 2.6: проектирование архитектуры и разработка ядра</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -32502,28 +32502,28 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Главный разработчик</t>
         </is>
       </c>
       <c r="E227" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="F227" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G227" t="n">
-        <v>350</v>
+        <v>286</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>ADTHPL-275</t>
+          <t>ADTHPL-278</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Интеграция с внешними SSP по OpenRTB 2.6: интеграция со смежными модулями платформы</t>
+          <t>Интеграция с внешними SSP по OpenRTB 2.6: техническое руководство разработкой и код-ревью</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -32533,28 +32533,28 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E228" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F228" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G228" t="n">
-        <v>350</v>
+        <v>297</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>ADTHPL-276</t>
+          <t>ADTHPL-279</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Интеграция с внешними SSP по OpenRTB 2.6: разработка хранения и обработки данных</t>
+          <t>Управление согласиями пользователей на обработку данных: разработка конвейера загрузки и обработки данных</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -32564,28 +32564,28 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Инженер данных</t>
         </is>
       </c>
       <c r="E229" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F229" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G229" t="n">
-        <v>350</v>
+        <v>294</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>ADTHPL-277</t>
+          <t>ADTHPL-282</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Интеграция с внешними SSP по OpenRTB 2.6: проектирование архитектуры и разработка ядра</t>
+          <t>Управление согласиями пользователей на обработку данных: техническое руководство разработкой и код-ревью</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -32595,28 +32595,28 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Главный разработчик</t>
+          <t>Руководитель команды</t>
         </is>
       </c>
       <c r="E230" t="n">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="F230" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G230" t="n">
-        <v>286</v>
+        <v>297</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>ADTHPL-278</t>
+          <t>ADTHPL-283</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Интеграция с внешними SSP по OpenRTB 2.6: техническое руководство разработкой и код-ревью</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: интеграция со смежными модулями платформы</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -32626,28 +32626,28 @@
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E231" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="F231" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G231" t="n">
-        <v>297</v>
+        <v>350</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>ADTHPL-279</t>
+          <t>ADTHPL-284</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: разработка конвейера загрузки и обработки данных</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: разработка хранения и обработки данных</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -32657,28 +32657,28 @@
       </c>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Инженер данных</t>
+          <t>Ведущий разработчик</t>
         </is>
       </c>
       <c r="E232" t="n">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="F232" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G232" t="n">
-        <v>294</v>
+        <v>350</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>ADTHPL-282</t>
+          <t>ADTHPL-285</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Управление согласиями пользователей на обработку данных: техническое руководство разработкой и код-ревью</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование архитектуры и разработка ядра</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
@@ -32688,28 +32688,28 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Руководитель команды</t>
+          <t>Главный разработчик</t>
         </is>
       </c>
       <c r="E233" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F233" t="n">
         <v>1</v>
       </c>
       <c r="G233" t="n">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>ADTHPL-283</t>
+          <t>ADTHPL-286</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: интеграция со смежными модулями платформы</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: разработка серверной части и API</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -32719,28 +32719,28 @@
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Главный разработчик</t>
         </is>
       </c>
       <c r="E234" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="F234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G234" t="n">
-        <v>350</v>
+        <v>294</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>ADTHPL-284</t>
+          <t>ADTHPL-287</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: разработка хранения и обработки данных</t>
+          <t>Кабинет селлера для самостоятельного запуска продвижения: разработка пользовательского интерфейса</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
@@ -32750,28 +32750,28 @@
       </c>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Ведущий разработчик</t>
+          <t>Главный разработчик</t>
         </is>
       </c>
       <c r="E235" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="F235" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G235" t="n">
-        <v>350</v>
+        <v>310</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>ADTHPL-285</t>
+          <t>ADTHPL-290</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: проектирование архитектуры и разработка ядра</t>
+          <t>Отчет sales lift по рекламной кампании: обучение и валидация модели</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -32781,59 +32781,59 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Главный разработчик</t>
+          <t>Ведущий специалист ML</t>
         </is>
       </c>
       <c r="E236" t="n">
-        <v>56</v>
+        <v>136</v>
       </c>
       <c r="F236" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G236" t="n">
-        <v>294</v>
+        <v>214</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>ADTHPL-286</t>
+          <t>ADTHPL-293</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: разработка серверной части и API</t>
+          <t>Сбор событий веб-витрины без сторонних cookies: исследование и формирование продуктовой гипотезы</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>CAPEX</t>
+          <t>OPEX</t>
         </is>
       </c>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Главный разработчик</t>
+          <t>Ведущий менеджер продукта</t>
         </is>
       </c>
       <c r="E237" t="n">
-        <v>56</v>
+        <v>140</v>
       </c>
       <c r="F237" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G237" t="n">
-        <v>294</v>
+        <v>210</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>ADTHPL-287</t>
+          <t>ADTHPL-295</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Кабинет селлера для самостоятельного запуска продвижения: разработка пользовательского интерфейса</t>
+          <t>Автоматическая передача в ОРД данных о показах и актах: анализ качества данных на тестовом контуре</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
@@ -32843,28 +32843,28 @@
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Главный разработчик</t>
+          <t>Аналитик данных</t>
         </is>
       </c>
       <c r="E238" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="F238" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G238" t="n">
-        <v>310</v>
+        <v>350</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>ADTHPL-290</t>
+          <t>ADTHPL-296</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Отчет sales lift по рекламной кампании: обучение и валидация модели</t>
+          <t>Автоматическая передача в ОРД данных о показах и актах: проверка расчета метрик</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -32874,140 +32874,47 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Ведущий специалист ML</t>
+          <t>Аналитик данных</t>
         </is>
       </c>
       <c r="E239" t="n">
-        <v>136</v>
+        <v>0</v>
       </c>
       <c r="F239" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G239" t="n">
-        <v>214</v>
+        <v>350</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>ADTHPL-293</t>
+          <t>ADTHPL-297</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Сбор событий веб-витрины без сторонних cookies: исследование и формирование продуктовой гипотезы</t>
+          <t>Автоматическая передача в ОРД данных о показах и актах: проектирование модели данных и витрин</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Ведущий менеджер продукта</t>
+          <t>Ведущий аналитик данных</t>
         </is>
       </c>
       <c r="E240" t="n">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="F240" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G240" t="n">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="241">
-      <c r="A241" t="inlineStr">
-        <is>
-          <t>ADTHPL-295</t>
-        </is>
-      </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>Автоматическая передача в ОРД данных о показах и актах: анализ качества данных на тестовом контуре</t>
-        </is>
-      </c>
-      <c r="C241" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>Аналитик данных</t>
-        </is>
-      </c>
-      <c r="E241" t="n">
-        <v>0</v>
-      </c>
-      <c r="F241" t="n">
-        <v>0</v>
-      </c>
-      <c r="G241" t="n">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" t="inlineStr">
-        <is>
-          <t>ADTHPL-296</t>
-        </is>
-      </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>Автоматическая передача в ОРД данных о показах и актах: проверка расчета метрик</t>
-        </is>
-      </c>
-      <c r="C242" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>Аналитик данных</t>
-        </is>
-      </c>
-      <c r="E242" t="n">
-        <v>0</v>
-      </c>
-      <c r="F242" t="n">
-        <v>0</v>
-      </c>
-      <c r="G242" t="n">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" t="inlineStr">
-        <is>
-          <t>ADTHPL-297</t>
-        </is>
-      </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>Автоматическая передача в ОРД данных о показах и актах: проектирование модели данных и витрин</t>
-        </is>
-      </c>
-      <c r="C243" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="D243" t="inlineStr">
-        <is>
-          <t>Ведущий аналитик данных</t>
-        </is>
-      </c>
-      <c r="E243" t="n">
-        <v>0</v>
-      </c>
-      <c r="F243" t="n">
-        <v>0</v>
-      </c>
-      <c r="G243" t="n">
         <v>350</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Timesheet AdTech Oct 2026: capitalize Gryada by role and catalog task
The Edtech lead developer role has CAPEX task ADTHPL-164 in the capitalization
phase in October; September OPEX was due only to the source comment, which is
absent in October. Now 100% CAPEX: 164 (120 h) + 168 of the same epic (56 h).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WUQDQoJZYHaVzbkcZbnkgZ
</commit_message>
<xml_diff>
--- a/out/Таймшит_AdTech_октябрь_2026_заполнен.xlsx
+++ b/out/Таймшит_AdTech_октябрь_2026_заполнен.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Были в сентябре" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лист1'!$A$1:$X$228</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Лист1'!$A$1:$X$229</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Были в сентябре'!$A$1:$L$37</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -735,7 +735,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X228"/>
+  <dimension ref="A1:X229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12.7109375" customWidth="1" min="1" max="7"/>
@@ -22986,14 +22986,14 @@
         <v>1</v>
       </c>
       <c r="N224" s="23" t="n">
-        <v>176</v>
+        <v>120</v>
       </c>
       <c r="O224" s="8" t="n"/>
       <c r="P224" s="27" t="n"/>
       <c r="Q224" s="27" t="n"/>
       <c r="R224" s="8" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="S224" s="8" t="inlineStr">
@@ -23003,12 +23003,12 @@
       </c>
       <c r="T224" s="8" t="inlineStr">
         <is>
-          <t>Сопровождение регулярной отчетности Эдтех: доработки и разбор обращений (4 кв. 2026)</t>
+          <t>Прогноз кликабельности для ранжирования ставок: мониторинг и логирование новой функциональности</t>
         </is>
       </c>
       <c r="U224" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-239</t>
+          <t>ADTHPL-164</t>
         </is>
       </c>
       <c r="V224" s="28" t="n">
@@ -23032,47 +23032,43 @@
       </c>
       <c r="C225" s="8" t="inlineStr">
         <is>
-          <t>CN-0981142</t>
+          <t>GK-0002680</t>
         </is>
       </c>
       <c r="D225" s="8" t="inlineStr">
         <is>
-          <t>Лошманов Александр Борисович</t>
+          <t>Гряда Игорь Леонидович</t>
         </is>
       </c>
       <c r="E225" s="8" t="inlineStr">
         <is>
-          <t>Инженер сопровождения</t>
+          <t>Ведущий разработчик проекта Эдтех</t>
         </is>
       </c>
       <c r="F225" s="8" t="inlineStr">
         <is>
-          <t>0f507677-229f-11f1-93e2-c4cbe1a36811</t>
+          <t>401c7277-4316-11e8-8109-5cf3fc374db0</t>
         </is>
       </c>
       <c r="G225" s="8" t="inlineStr">
         <is>
-          <t>c0029a41-22a0-11f1-93e2-c4cbe1a36811</t>
+          <t>512cec66-1cb6-11ef-ab4e-f8f21e64b171</t>
         </is>
       </c>
       <c r="H225" s="8" t="inlineStr">
         <is>
-          <t>loshmanov_ab@magnit.ru</t>
-        </is>
-      </c>
-      <c r="I225" s="8" t="inlineStr">
-        <is>
-          <t>Департамент по развитию и разработке онлайн платформ</t>
-        </is>
-      </c>
+          <t>gryada_il@magnit.ru</t>
+        </is>
+      </c>
+      <c r="I225" s="8" t="n"/>
       <c r="J225" s="8" t="inlineStr">
         <is>
-          <t>Науменко Андрей Викторович</t>
+          <t>Моисеенко Ярослав Александрович</t>
         </is>
       </c>
       <c r="K225" s="8" t="inlineStr">
         <is>
-          <t>Команда развития медиаконтента</t>
+          <t>Сектор разработки регулярной отчётности</t>
         </is>
       </c>
       <c r="L225" s="23" t="inlineStr">
@@ -23084,14 +23080,14 @@
         <v>1</v>
       </c>
       <c r="N225" s="23" t="n">
-        <v>176</v>
+        <v>56</v>
       </c>
       <c r="O225" s="8" t="n"/>
       <c r="P225" s="27" t="n"/>
       <c r="Q225" s="27" t="n"/>
       <c r="R225" s="8" t="inlineStr">
         <is>
-          <t>OPEX</t>
+          <t>CAPEX</t>
         </is>
       </c>
       <c r="S225" s="8" t="inlineStr">
@@ -23101,12 +23097,12 @@
       </c>
       <c r="T225" s="8" t="inlineStr">
         <is>
-          <t>Сопровождение промышленной эксплуатации партнерской платформы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
+          <t>Прогноз кликабельности для ранжирования ставок: разработка серверной части и API</t>
         </is>
       </c>
       <c r="U225" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-235</t>
+          <t>ADTHPL-168</t>
         </is>
       </c>
       <c r="V225" s="28" t="n">
@@ -23130,47 +23126,47 @@
       </c>
       <c r="C226" s="8" t="inlineStr">
         <is>
-          <t>CN-0744573</t>
+          <t>CN-0981142</t>
         </is>
       </c>
       <c r="D226" s="8" t="inlineStr">
         <is>
-          <t>Ардаширов Денис Тимурович</t>
+          <t>Лошманов Александр Борисович</t>
         </is>
       </c>
       <c r="E226" s="8" t="inlineStr">
         <is>
-          <t>Директор департамента</t>
+          <t>Инженер сопровождения</t>
         </is>
       </c>
       <c r="F226" s="8" t="inlineStr">
         <is>
-          <t>8b6edcd4-c45f-11ef-ab50-f8f21e64b170</t>
+          <t>0f507677-229f-11f1-93e2-c4cbe1a36811</t>
         </is>
       </c>
       <c r="G226" s="8" t="inlineStr">
         <is>
-          <t>8b6edd55-c45f-11ef-ab50-f8f21e64b170</t>
+          <t>c0029a41-22a0-11f1-93e2-c4cbe1a36811</t>
         </is>
       </c>
       <c r="H226" s="8" t="inlineStr">
         <is>
-          <t>ardashirov@magnit.ru</t>
+          <t>loshmanov_ab@magnit.ru</t>
         </is>
       </c>
       <c r="I226" s="8" t="inlineStr">
         <is>
-          <t>Департамент продуктов коммерции и механики рекламных технологий</t>
+          <t>Департамент по развитию и разработке онлайн платформ</t>
         </is>
       </c>
       <c r="J226" s="8" t="inlineStr">
         <is>
-          <t>Марлье Людмила Анатольевна</t>
+          <t>Науменко Андрей Викторович</t>
         </is>
       </c>
       <c r="K226" s="8" t="inlineStr">
         <is>
-          <t>Бизнес-формат Рекламные технологии</t>
+          <t>Команда развития медиаконтента</t>
         </is>
       </c>
       <c r="L226" s="23" t="inlineStr">
@@ -23194,17 +23190,17 @@
       </c>
       <c r="S226" s="8" t="inlineStr">
         <is>
-          <t>Менеджмент/ Административные задачи</t>
+          <t>Разработка (кодирование) ПО</t>
         </is>
       </c>
       <c r="T226" s="8" t="inlineStr">
         <is>
-          <t>Стратегическое управление департаментом и бюджетирование (4 кв. 2026)</t>
+          <t>Сопровождение промышленной эксплуатации партнерской платформы: мониторинг, инциденты, обновления (4 кв. 2026)</t>
         </is>
       </c>
       <c r="U226" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-242</t>
+          <t>ADTHPL-235</t>
         </is>
       </c>
       <c r="V226" s="28" t="n">
@@ -23218,7 +23214,7 @@
     <row r="227">
       <c r="A227" s="8" t="inlineStr">
         <is>
-          <t>Аналитика</t>
+          <t>Бизнес</t>
         </is>
       </c>
       <c r="B227" s="8" t="inlineStr">
@@ -23228,100 +23224,90 @@
       </c>
       <c r="C227" s="8" t="inlineStr">
         <is>
-          <t>CN-1090167</t>
+          <t>CN-0744573</t>
         </is>
       </c>
       <c r="D227" s="8" t="inlineStr">
         <is>
-          <t>Чижиков Никита Игоревич</t>
+          <t>Ардаширов Денис Тимурович</t>
         </is>
       </c>
       <c r="E227" s="8" t="inlineStr">
         <is>
-          <t>Специалист ML</t>
+          <t>Директор департамента</t>
         </is>
       </c>
       <c r="F227" s="8" t="inlineStr">
         <is>
-          <t>664a7fef-c2e6-11f1-86a6-3a68dd8b748f</t>
+          <t>8b6edcd4-c45f-11ef-ab50-f8f21e64b170</t>
         </is>
       </c>
       <c r="G227" s="8" t="inlineStr">
         <is>
-          <t>fd95a41a-c2e6-11f1-86a6-3a68dd8b748f</t>
+          <t>8b6edd55-c45f-11ef-ab50-f8f21e64b170</t>
         </is>
       </c>
       <c r="H227" s="8" t="inlineStr">
         <is>
-          <t>chizhikov_ni@magnit.ru</t>
+          <t>ardashirov@magnit.ru</t>
         </is>
       </c>
       <c r="I227" s="8" t="inlineStr">
         <is>
-          <t>Департамент по управлению данными и операционной аналитике цифровых платформ</t>
+          <t>Департамент продуктов коммерции и механики рекламных технологий</t>
         </is>
       </c>
       <c r="J227" s="8" t="inlineStr">
         <is>
-          <t>Соловьев Никита Александрович</t>
+          <t>Марлье Людмила Анатольевна</t>
         </is>
       </c>
       <c r="K227" s="8" t="inlineStr">
         <is>
-          <t>Команда машинного обучения в рекламных технологиях</t>
+          <t>Бизнес-формат Рекламные технологии</t>
         </is>
       </c>
       <c r="L227" s="23" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>да</t>
         </is>
       </c>
       <c r="M227" s="23" t="n">
         <v>1</v>
       </c>
       <c r="N227" s="23" t="n">
-        <v>88</v>
-      </c>
-      <c r="O227" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="P227" s="27" t="n">
+        <v>176</v>
+      </c>
+      <c r="O227" s="8" t="n"/>
+      <c r="P227" s="27" t="n"/>
+      <c r="Q227" s="27" t="n"/>
+      <c r="R227" s="8" t="inlineStr">
+        <is>
+          <t>OPEX</t>
+        </is>
+      </c>
+      <c r="S227" s="8" t="inlineStr">
+        <is>
+          <t>Менеджмент/ Административные задачи</t>
+        </is>
+      </c>
+      <c r="T227" s="8" t="inlineStr">
+        <is>
+          <t>Стратегическое управление департаментом и бюджетирование (4 кв. 2026)</t>
+        </is>
+      </c>
+      <c r="U227" s="8" t="inlineStr">
+        <is>
+          <t>ADTHPL-242</t>
+        </is>
+      </c>
+      <c r="V227" s="28" t="n">
         <v>46296</v>
-      </c>
-      <c r="Q227" s="27" t="n">
-        <v>46306</v>
-      </c>
-      <c r="R227" s="8" t="inlineStr">
-        <is>
-          <t>CAPEX</t>
-        </is>
-      </c>
-      <c r="S227" s="8" t="inlineStr">
-        <is>
-          <t>Разработка (кодирование) ПО</t>
-        </is>
-      </c>
-      <c r="T227" s="8" t="inlineStr">
-        <is>
-          <t>Дашборд эффективности кампаний в реальном времени: обучение и валидация модели</t>
-        </is>
-      </c>
-      <c r="U227" s="8" t="inlineStr">
-        <is>
-          <t>ADTHPL-147</t>
-        </is>
-      </c>
-      <c r="V227" s="28" t="n">
-        <v>46307</v>
       </c>
       <c r="W227" s="28" t="n">
         <v>46326</v>
       </c>
-      <c r="X227" s="8" t="inlineStr">
-        <is>
-          <t>приступили к работе в октябре</t>
-        </is>
-      </c>
+      <c r="X227" s="8" t="n"/>
     </row>
     <row r="228">
       <c r="A228" s="8" t="inlineStr">
@@ -23388,7 +23374,7 @@
         <v>1</v>
       </c>
       <c r="N228" s="23" t="n">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="O228" s="8" t="n">
         <v>7</v>
@@ -23411,16 +23397,16 @@
       </c>
       <c r="T228" s="8" t="inlineStr">
         <is>
-          <t>Отчет sales lift по рекламной кампании: обучение и валидация модели</t>
+          <t>Дашборд эффективности кампаний в реальном времени: обучение и валидация модели</t>
         </is>
       </c>
       <c r="U228" s="8" t="inlineStr">
         <is>
-          <t>ADTHPL-290</t>
+          <t>ADTHPL-147</t>
         </is>
       </c>
       <c r="V228" s="28" t="n">
-        <v>46314</v>
+        <v>46307</v>
       </c>
       <c r="W228" s="28" t="n">
         <v>46326</v>
@@ -23431,8 +23417,116 @@
         </is>
       </c>
     </row>
+    <row r="229">
+      <c r="A229" s="8" t="inlineStr">
+        <is>
+          <t>Аналитика</t>
+        </is>
+      </c>
+      <c r="B229" s="8" t="inlineStr">
+        <is>
+          <t>AdTech</t>
+        </is>
+      </c>
+      <c r="C229" s="8" t="inlineStr">
+        <is>
+          <t>CN-1090167</t>
+        </is>
+      </c>
+      <c r="D229" s="8" t="inlineStr">
+        <is>
+          <t>Чижиков Никита Игоревич</t>
+        </is>
+      </c>
+      <c r="E229" s="8" t="inlineStr">
+        <is>
+          <t>Специалист ML</t>
+        </is>
+      </c>
+      <c r="F229" s="8" t="inlineStr">
+        <is>
+          <t>664a7fef-c2e6-11f1-86a6-3a68dd8b748f</t>
+        </is>
+      </c>
+      <c r="G229" s="8" t="inlineStr">
+        <is>
+          <t>fd95a41a-c2e6-11f1-86a6-3a68dd8b748f</t>
+        </is>
+      </c>
+      <c r="H229" s="8" t="inlineStr">
+        <is>
+          <t>chizhikov_ni@magnit.ru</t>
+        </is>
+      </c>
+      <c r="I229" s="8" t="inlineStr">
+        <is>
+          <t>Департамент по управлению данными и операционной аналитике цифровых платформ</t>
+        </is>
+      </c>
+      <c r="J229" s="8" t="inlineStr">
+        <is>
+          <t>Соловьев Никита Александрович</t>
+        </is>
+      </c>
+      <c r="K229" s="8" t="inlineStr">
+        <is>
+          <t>Команда машинного обучения в рекламных технологиях</t>
+        </is>
+      </c>
+      <c r="L229" s="23" t="inlineStr">
+        <is>
+          <t>нет</t>
+        </is>
+      </c>
+      <c r="M229" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="N229" s="23" t="n">
+        <v>32</v>
+      </c>
+      <c r="O229" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="P229" s="27" t="n">
+        <v>46296</v>
+      </c>
+      <c r="Q229" s="27" t="n">
+        <v>46306</v>
+      </c>
+      <c r="R229" s="8" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="S229" s="8" t="inlineStr">
+        <is>
+          <t>Разработка (кодирование) ПО</t>
+        </is>
+      </c>
+      <c r="T229" s="8" t="inlineStr">
+        <is>
+          <t>Отчет sales lift по рекламной кампании: обучение и валидация модели</t>
+        </is>
+      </c>
+      <c r="U229" s="8" t="inlineStr">
+        <is>
+          <t>ADTHPL-290</t>
+        </is>
+      </c>
+      <c r="V229" s="28" t="n">
+        <v>46314</v>
+      </c>
+      <c r="W229" s="28" t="n">
+        <v>46326</v>
+      </c>
+      <c r="X229" s="8" t="inlineStr">
+        <is>
+          <t>приступили к работе в октябре</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:X228"/>
+  <autoFilter ref="A1:X229"/>
   <conditionalFormatting sqref="D1:D105 D107:D1048576">
     <cfRule type="duplicateValues" priority="9" dxfId="0"/>
   </conditionalFormatting>

</xml_diff>